<commit_message>
added some more functions
</commit_message>
<xml_diff>
--- a/excel 5 functions 30-07-2026.xlsx
+++ b/excel 5 functions 30-07-2026.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell\Documents\excel_wise-owl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B641FA4E-7575-4720-8E05-95293311CD38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90D22E15-C163-4938-BD04-1E7E3A57F4ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="today" sheetId="1" r:id="rId1"/>
     <sheet name="now" sheetId="2" r:id="rId2"/>
     <sheet name="dateif" sheetId="3" r:id="rId3"/>
+    <sheet name="year , month, day" sheetId="5" r:id="rId4"/>
+    <sheet name="workday" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>to write todays date</t>
   </si>
@@ -89,6 +91,27 @@
   </si>
   <si>
     <t>Calculate total months.</t>
+  </si>
+  <si>
+    <t>Delivery after 7 working days.</t>
+  </si>
+  <si>
+    <t>Project completion after 20 working days.</t>
+  </si>
+  <si>
+    <t>Find the date 5 working days before today.</t>
+  </si>
+  <si>
+    <t>Extract the year.</t>
+  </si>
+  <si>
+    <t>Extract the month.</t>
+  </si>
+  <si>
+    <t>Extract the day.</t>
+  </si>
+  <si>
+    <t>Calculate total days.</t>
   </si>
 </sst>
 </file>
@@ -132,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -142,6 +165,8 @@
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="15" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -422,37 +447,38 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A5:F9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="1">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1">
         <f ca="1">TODAY()</f>
         <v>46233</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <f ca="1">DATE(2026,12,31)-TODAY()</f>
-        <v>154</v>
-      </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="str">
+      <c r="F7" t="str">
         <f ca="1">IF(A2&lt;TODAY(),"Yes","No")</f>
         <v>Yes</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>1</v>
+      </c>
+      <c r="F9" t="str">
+        <f ca="1">IF(A2&lt;TODAY(),"Yes","No")</f>
+        <v>Yes</v>
       </c>
     </row>
   </sheetData>
@@ -474,7 +500,7 @@
       </c>
       <c r="E1" s="2">
         <f ca="1">NOW()</f>
-        <v>46233.376940972223</v>
+        <v>46233.847805902777</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -483,7 +509,7 @@
       </c>
       <c r="E2" s="2">
         <f ca="1">NOW()</f>
-        <v>46233.376940972223</v>
+        <v>46233.847805902777</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -492,7 +518,7 @@
       </c>
       <c r="E3" s="2">
         <f ca="1">NOW()</f>
-        <v>46233.376940972223</v>
+        <v>46233.847805902777</v>
       </c>
     </row>
   </sheetData>
@@ -502,7 +528,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D021B7EF-C2F1-4F0E-9A57-227B7CB45B29}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
@@ -537,6 +563,102 @@
         <v>54</v>
       </c>
     </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <f>DATEDIF(H2,I2,"D")</f>
+        <v>1662</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D324E5E-FEC4-4119-B923-66997D4E9948}">
+  <dimension ref="A2:C8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="5">
+        <v>46381</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4">
+        <f>YEAR(A2)</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6">
+        <f>MONTH(A2)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8">
+        <f>DAY(A2)</f>
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F43B13C4-5876-4A49-B7FE-E28C0A80B1F0}">
+  <dimension ref="A2:E8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="6">
+        <v>46233</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4">
+        <f>WORKDAY(A2,7)</f>
+        <v>46244</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6">
+        <f>WORKDAY(A2,20)</f>
+        <v>46261</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8">
+        <f ca="1">WORKDAY(TODAY(),-5)</f>
+        <v>46226</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>